<commit_message>
Cleaned up homepage layout, nav menu, DetailsFourthAnnual page, and updated Players spreadsheet
</commit_message>
<xml_diff>
--- a/UConnBleedBlue/wwwroot/Data/PlayersForTesting.xlsx
+++ b/UConnBleedBlue/wwwroot/Data/PlayersForTesting.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\UConnBleedBlue\UConnBleedBlue\wwwroot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1198515-B20B-4A50-9A6E-731B60619DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EDF8018-767E-4A08-8AFD-84F894890622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2325" windowWidth="38640" windowHeight="21120" xr2:uid="{4F83266A-41F9-4FA3-9290-1EB5622BBFC1}"/>
+    <workbookView xWindow="33060" yWindow="3495" windowWidth="21600" windowHeight="13770" xr2:uid="{4F83266A-41F9-4FA3-9290-1EB5622BBFC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Demers, Kenny</t>
   </si>
@@ -499,44 +499,10 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1969</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="1">
-        <v>2</v>
-      </c>
+      <c r="B3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1969</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1">
-        <v>2</v>
-      </c>
+      <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
@@ -1048,10 +1014,8 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{D4F421DD-A322-4F00-A209-B464A28664A6}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{F3A9F971-DAE7-49EC-84DE-5020AB7D35F8}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{DFF9F2B3-4F7F-4233-BB59-BF5F0C6C0891}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>